<commit_message>
Add admin panel, response shortcuts, and chat UI improvements
- Add /admin route with admin.html dashboard template
- Add admin API endpoints for user conversation history and activity stats
- Expand response_processor with shortcut detection for common queries (week, KP weight, item lookup)
- Fix suggestion handling to use shortcut-generated suggestions when available
- Update chat_enhanced.html UI tweaks
- Update Sales Email login data

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/User_login/Sales Email Update.xlsx
+++ b/User_login/Sales Email Update.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\vscode\powerbi_api\User_login\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\vscode\Chatbot\User_login\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82218F58-8AE4-4E4B-9D07-C78DA55507D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F0DDFBA-AD26-4B59-8729-EF953C0CD90B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="1" activeTab="1" xr2:uid="{64160F79-1A7E-4E2D-B1AE-60ABFC61A377}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{64160F79-1A7E-4E2D-B1AE-60ABFC61A377}"/>
   </bookViews>
   <sheets>
     <sheet name="List Users-SCM" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="377" uniqueCount="243">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="385" uniqueCount="247">
   <si>
     <t>USER_ID</t>
   </si>
@@ -859,12 +859,24 @@
   <si>
     <t>Test@nanyangtextile.com</t>
   </si>
+  <si>
+    <t>wicharit.l@nanyangtextile.com</t>
+  </si>
+  <si>
+    <t>WICHARIT.L</t>
+  </si>
+  <si>
+    <t>tatsanee.s@nanyangtextile.com</t>
+  </si>
+  <si>
+    <t>TATSANEE.S</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -903,6 +915,12 @@
       <family val="2"/>
       <charset val="222"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -947,7 +965,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -991,6 +1009,8 @@
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1326,15 +1346,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EDED9074-41CC-4D78-9FCD-68DC80C75AC5}">
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:F45"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.19921875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.19921875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.796875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="8.5" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="32.09765625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.69921875" style="2" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.5" customWidth="1"/>
+    <col min="5" max="5" width="16.5" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.3984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -1681,7 +1701,7 @@
       </c>
       <c r="F19" s="9"/>
     </row>
-    <row r="20" spans="1:6" ht="45.6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" ht="34.200000000000003" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
         <v>56</v>
       </c>
@@ -1699,7 +1719,226 @@
       </c>
       <c r="F20" s="9"/>
     </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" s="4" t="s">
+        <v>244</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D21" s="20" t="s">
+        <v>243</v>
+      </c>
+      <c r="E21" s="5"/>
+      <c r="F21" s="9"/>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" s="4" t="s">
+        <v>246</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D22" s="19" t="s">
+        <v>245</v>
+      </c>
+      <c r="E22" s="5"/>
+      <c r="F22" s="9"/>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" s="4"/>
+      <c r="B23" s="4"/>
+      <c r="C23" s="4"/>
+      <c r="D23" s="4"/>
+      <c r="E23" s="5"/>
+      <c r="F23" s="9"/>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" s="4"/>
+      <c r="B24" s="4"/>
+      <c r="C24" s="4"/>
+      <c r="D24" s="4"/>
+      <c r="E24" s="5"/>
+      <c r="F24" s="9"/>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" s="4"/>
+      <c r="B25" s="4"/>
+      <c r="C25" s="4"/>
+      <c r="D25" s="4"/>
+      <c r="E25" s="5"/>
+      <c r="F25" s="9"/>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" s="4"/>
+      <c r="B26" s="4"/>
+      <c r="C26" s="4"/>
+      <c r="D26" s="4"/>
+      <c r="E26" s="5"/>
+      <c r="F26" s="9"/>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" s="4"/>
+      <c r="B27" s="4"/>
+      <c r="C27" s="4"/>
+      <c r="D27" s="4"/>
+      <c r="E27" s="5"/>
+      <c r="F27" s="9"/>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" s="4"/>
+      <c r="B28" s="4"/>
+      <c r="C28" s="4"/>
+      <c r="D28" s="4"/>
+      <c r="E28" s="5"/>
+      <c r="F28" s="9"/>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" s="4"/>
+      <c r="B29" s="4"/>
+      <c r="C29" s="4"/>
+      <c r="D29" s="4"/>
+      <c r="E29" s="5"/>
+      <c r="F29" s="9"/>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" s="4"/>
+      <c r="B30" s="4"/>
+      <c r="C30" s="4"/>
+      <c r="D30" s="4"/>
+      <c r="E30" s="5"/>
+      <c r="F30" s="9"/>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" s="4"/>
+      <c r="B31" s="4"/>
+      <c r="C31" s="4"/>
+      <c r="D31" s="4"/>
+      <c r="E31" s="5"/>
+      <c r="F31" s="9"/>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" s="4"/>
+      <c r="B32" s="4"/>
+      <c r="C32" s="4"/>
+      <c r="D32" s="4"/>
+      <c r="E32" s="5"/>
+      <c r="F32" s="9"/>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" s="4"/>
+      <c r="B33" s="4"/>
+      <c r="C33" s="4"/>
+      <c r="D33" s="4"/>
+      <c r="E33" s="5"/>
+      <c r="F33" s="9"/>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" s="4"/>
+      <c r="B34" s="4"/>
+      <c r="C34" s="4"/>
+      <c r="D34" s="4"/>
+      <c r="E34" s="5"/>
+      <c r="F34" s="9"/>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" s="4"/>
+      <c r="B35" s="4"/>
+      <c r="C35" s="4"/>
+      <c r="D35" s="4"/>
+      <c r="E35" s="5"/>
+      <c r="F35" s="9"/>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" s="4"/>
+      <c r="B36" s="4"/>
+      <c r="C36" s="4"/>
+      <c r="D36" s="4"/>
+      <c r="E36" s="5"/>
+      <c r="F36" s="9"/>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" s="4"/>
+      <c r="B37" s="4"/>
+      <c r="C37" s="4"/>
+      <c r="D37" s="4"/>
+      <c r="E37" s="5"/>
+      <c r="F37" s="9"/>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" s="4"/>
+      <c r="B38" s="4"/>
+      <c r="C38" s="4"/>
+      <c r="D38" s="4"/>
+      <c r="E38" s="5"/>
+      <c r="F38" s="9"/>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" s="4"/>
+      <c r="B39" s="4"/>
+      <c r="C39" s="4"/>
+      <c r="D39" s="4"/>
+      <c r="E39" s="5"/>
+      <c r="F39" s="9"/>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" s="4"/>
+      <c r="B40" s="4"/>
+      <c r="C40" s="4"/>
+      <c r="D40" s="4"/>
+      <c r="E40" s="5"/>
+      <c r="F40" s="9"/>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" s="4"/>
+      <c r="B41" s="4"/>
+      <c r="C41" s="4"/>
+      <c r="D41" s="4"/>
+      <c r="E41" s="5"/>
+      <c r="F41" s="9"/>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" s="4"/>
+      <c r="B42" s="4"/>
+      <c r="C42" s="4"/>
+      <c r="D42" s="4"/>
+      <c r="E42" s="5"/>
+      <c r="F42" s="9"/>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" s="4"/>
+      <c r="B43" s="4"/>
+      <c r="C43" s="4"/>
+      <c r="D43" s="4"/>
+      <c r="E43" s="5"/>
+      <c r="F43" s="9"/>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" s="4"/>
+      <c r="B44" s="4"/>
+      <c r="C44" s="4"/>
+      <c r="D44" s="4"/>
+      <c r="E44" s="5"/>
+      <c r="F44" s="9"/>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" s="4"/>
+      <c r="B45" s="4"/>
+      <c r="C45" s="4"/>
+      <c r="D45" s="4"/>
+      <c r="E45" s="5"/>
+      <c r="F45" s="9"/>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D21" r:id="rId1" xr:uid="{9EF5377D-3577-474F-87D9-3DF903E90C2B}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Fix CSRF headers on all fetch requests, refine no-repeat rule, reorder note output
- Add X-CSRFToken header to all POST/PUT/DELETE fetch calls in admin.html and chat_enhanced.html
- Clarify anti-repeat rule in response_processor.py: focus on current message only, forbid bundling old answers
- Move footnote (note) to end of tool output instead of prepending it
- Update Sales Email spreadsheet

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/User_login/Sales Email Update.xlsx
+++ b/User_login/Sales Email Update.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\vscode\Chatbot\User_login\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F0DDFBA-AD26-4B59-8729-EF953C0CD90B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{348CCD72-3E82-476C-9066-3AC80A0BA56A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{64160F79-1A7E-4E2D-B1AE-60ABFC61A377}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="385" uniqueCount="247">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="389" uniqueCount="249">
   <si>
     <t>USER_ID</t>
   </si>
@@ -870,6 +870,12 @@
   </si>
   <si>
     <t>TATSANEE.S</t>
+  </si>
+  <si>
+    <t>kampanart.w</t>
+  </si>
+  <si>
+    <t>kampanart.w@nanyangtextile.com</t>
   </si>
 </sst>
 </file>
@@ -1752,10 +1758,18 @@
       <c r="F22" s="9"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A23" s="4"/>
-      <c r="B23" s="4"/>
-      <c r="C23" s="4"/>
-      <c r="D23" s="4"/>
+      <c r="A23" t="s">
+        <v>247</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D23" t="s">
+        <v>248</v>
+      </c>
       <c r="E23" s="5"/>
       <c r="F23" s="9"/>
     </row>

</xml_diff>

<commit_message>
Tighten chat rate limit to 5 msg/min with per-bucket windows
- rate_limit: chat bucket now uses 60s window (5 msgs/min) instead of shared 300s window
- rate_limit: add _RATE_WINDOW_BY_BUCKET for per-bucket time window config
- deploy: add rate_limit.py to deploy file list to prevent container crash-loop
- chat UI: capture confirm modal callback before closing to fix potential race condition
- tests: update window expiry test to use per-bucket window

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/User_login/Sales Email Update.xlsx
+++ b/User_login/Sales Email Update.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\vscode\Chatbot\User_login\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{348CCD72-3E82-476C-9066-3AC80A0BA56A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E20F49E-848F-4E76-87CB-E109C2DADCAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{64160F79-1A7E-4E2D-B1AE-60ABFC61A377}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="389" uniqueCount="249">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="397" uniqueCount="253">
   <si>
     <t>USER_ID</t>
   </si>
@@ -872,10 +872,22 @@
     <t>TATSANEE.S</t>
   </si>
   <si>
-    <t>kampanart.w</t>
-  </si>
-  <si>
     <t>kampanart.w@nanyangtextile.com</t>
+  </si>
+  <si>
+    <t>Kampanart.w</t>
+  </si>
+  <si>
+    <t>poomipat.c@nanyangtextile.com</t>
+  </si>
+  <si>
+    <t>Poomipat.c</t>
+  </si>
+  <si>
+    <t>patchara.c@nanyangtextile.com</t>
+  </si>
+  <si>
+    <t>Patchara.c</t>
   </si>
 </sst>
 </file>
@@ -971,7 +983,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1017,6 +1029,9 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" quotePrefix="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1352,7 +1367,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EDED9074-41CC-4D78-9FCD-68DC80C75AC5}">
-  <dimension ref="A1:F45"/>
+  <dimension ref="A1:F43"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.19921875" bestFit="1" customWidth="1"/>
@@ -1759,7 +1774,7 @@
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="B23" s="4" t="s">
         <v>7</v>
@@ -1768,24 +1783,40 @@
         <v>8</v>
       </c>
       <c r="D23" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="E23" s="5"/>
       <c r="F23" s="9"/>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A24" s="4"/>
-      <c r="B24" s="4"/>
-      <c r="C24" s="4"/>
-      <c r="D24" s="4"/>
+      <c r="A24" s="4" t="s">
+        <v>250</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D24" s="21" t="s">
+        <v>249</v>
+      </c>
       <c r="E24" s="5"/>
       <c r="F24" s="9"/>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A25" s="4"/>
-      <c r="B25" s="4"/>
-      <c r="C25" s="4"/>
-      <c r="D25" s="4"/>
+      <c r="A25" s="4" t="s">
+        <v>252</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D25" s="4" t="s">
+        <v>251</v>
+      </c>
       <c r="E25" s="5"/>
       <c r="F25" s="9"/>
     </row>
@@ -1933,25 +1964,10 @@
       <c r="E43" s="5"/>
       <c r="F43" s="9"/>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A44" s="4"/>
-      <c r="B44" s="4"/>
-      <c r="C44" s="4"/>
-      <c r="D44" s="4"/>
-      <c r="E44" s="5"/>
-      <c r="F44" s="9"/>
-    </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A45" s="4"/>
-      <c r="B45" s="4"/>
-      <c r="C45" s="4"/>
-      <c r="D45" s="4"/>
-      <c r="E45" s="5"/>
-      <c r="F45" s="9"/>
-    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="D21" r:id="rId1" xr:uid="{9EF5377D-3577-474F-87D9-3DF903E90C2B}"/>
+    <hyperlink ref="D24" r:id="rId2" xr:uid="{2A2E1194-9AD0-43A3-8861-A9E858B6CE8A}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>